<commit_message>
fix: correct WBS milestone description (6주→7주) and UX doc date (2020→2026)
</commit_message>
<xml_diff>
--- a/LifeLog_WBS.xlsx
+++ b/LifeLog_WBS.xlsx
@@ -2972,19 +2972,19 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>WP1-1</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ├ W1 — 파일럿 기관 현장 인터뷰</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="n"/>
+          <t>WP1-3</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├ W4 — UI/UX 상세 설계 + WBS 작성</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
@@ -3010,19 +3010,19 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>WP1-3</t>
+          <t>WP1-2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W4 — UI/UX 상세 설계 + WBS 작성</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
+          <t xml:space="preserve">  ├ W2~W3 — 요구사항 정제 + PRD 확정 + 기술아키텍처 + 데이터/DB/API 설계</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
       <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
@@ -3048,17 +3048,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>WP1-2</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ├ W2~W3 — 요구사항 정제 + PRD 확정 + 기술아키텍처 + 데이터/DB/API 설계</t>
+          <t>WP1-1</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├ W1 — 파일럿 기관 현장 인터뷰</t>
         </is>
       </c>
       <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
@@ -3086,29 +3086,29 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>WP2-2</t>
+          <t>WP2-1</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W7~W13 — 핵심 기능 개발</t>
+          <t xml:space="preserve">  ├ W5~W6 — 개발환경설정</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
       <c r="I10" s="10" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="10" t="n"/>
-      <c r="L10" s="10" t="n"/>
-      <c r="M10" s="10" t="n"/>
-      <c r="N10" s="10" t="n"/>
-      <c r="O10" s="10" t="n"/>
-      <c r="P10" s="10" t="n"/>
-      <c r="Q10" s="10" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
+      <c r="Q10" s="6" t="n"/>
       <c r="R10" s="6" t="n"/>
       <c r="S10" s="6" t="n"/>
       <c r="T10" s="6" t="n"/>
@@ -3124,29 +3124,29 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>WP2-1</t>
+          <t>WP2-2</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W5~W6 — 개발환경설정</t>
+          <t xml:space="preserve">  ├ W7~W13 — 핵심 기능 개발</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
       <c r="I11" s="10" t="n"/>
-      <c r="J11" s="6" t="n"/>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="n"/>
-      <c r="O11" s="6" t="n"/>
-      <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="6" t="n"/>
+      <c r="J11" s="10" t="n"/>
+      <c r="K11" s="10" t="n"/>
+      <c r="L11" s="10" t="n"/>
+      <c r="M11" s="10" t="n"/>
+      <c r="N11" s="10" t="n"/>
+      <c r="O11" s="10" t="n"/>
+      <c r="P11" s="10" t="n"/>
+      <c r="Q11" s="10" t="n"/>
       <c r="R11" s="6" t="n"/>
       <c r="S11" s="6" t="n"/>
       <c r="T11" s="6" t="n"/>
@@ -3200,12 +3200,12 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>WP3-1</t>
+          <t>WP3-3</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W17 — PoC 운영 (1차 주)</t>
+          <t xml:space="preserve">  ├ W19 — PoC 최종 평가 + 의견수렴</t>
         </is>
       </c>
       <c r="C13" s="8" t="n"/>
@@ -3225,10 +3225,10 @@
       <c r="Q13" s="8" t="n"/>
       <c r="R13" s="8" t="n"/>
       <c r="S13" s="8" t="n"/>
-      <c r="T13" s="10" t="n"/>
-      <c r="U13" s="10" t="n"/>
-      <c r="V13" s="8" t="n"/>
-      <c r="W13" s="8" t="n"/>
+      <c r="T13" s="8" t="n"/>
+      <c r="U13" s="8" t="n"/>
+      <c r="V13" s="10" t="n"/>
+      <c r="W13" s="10" t="n"/>
       <c r="X13" s="8" t="n"/>
       <c r="Y13" s="8" t="n"/>
       <c r="Z13" s="8" t="n"/>
@@ -3238,12 +3238,12 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>WP3-3</t>
+          <t>WP3-1</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W19 — PoC 최종 평가 + 의견수렴</t>
+          <t xml:space="preserve">  ├ W17 — PoC 운영 (1차 주)</t>
         </is>
       </c>
       <c r="C14" s="8" t="n"/>
@@ -3263,10 +3263,10 @@
       <c r="Q14" s="8" t="n"/>
       <c r="R14" s="8" t="n"/>
       <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
-      <c r="U14" s="8" t="n"/>
-      <c r="V14" s="10" t="n"/>
-      <c r="W14" s="10" t="n"/>
+      <c r="T14" s="10" t="n"/>
+      <c r="U14" s="10" t="n"/>
+      <c r="V14" s="8" t="n"/>
+      <c r="W14" s="8" t="n"/>
       <c r="X14" s="8" t="n"/>
       <c r="Y14" s="8" t="n"/>
       <c r="Z14" s="8" t="n"/>
@@ -3390,12 +3390,12 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>WP4-2</t>
+          <t>WP4-1</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W22 — 안정화 테스트</t>
+          <t xml:space="preserve">  ├ W21 — 보완 개발</t>
         </is>
       </c>
       <c r="C18" s="9" t="n"/>
@@ -3419,21 +3419,21 @@
       <c r="U18" s="9" t="n"/>
       <c r="V18" s="9" t="n"/>
       <c r="W18" s="9" t="n"/>
-      <c r="X18" s="9" t="n"/>
+      <c r="X18" s="10" t="n"/>
       <c r="Y18" s="10" t="n"/>
-      <c r="Z18" s="10" t="n"/>
+      <c r="Z18" s="9" t="n"/>
       <c r="AA18" s="9" t="n"/>
       <c r="AB18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>WP4-4</t>
+          <t>WP4-2</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W24 — 프로덕션 배포 + 최종 QA + 프로젝트 종료</t>
+          <t xml:space="preserve">  ├ W22 — 안정화 테스트</t>
         </is>
       </c>
       <c r="C19" s="9" t="n"/>
@@ -3458,20 +3458,20 @@
       <c r="V19" s="9" t="n"/>
       <c r="W19" s="9" t="n"/>
       <c r="X19" s="9" t="n"/>
-      <c r="Y19" s="9" t="n"/>
-      <c r="Z19" s="9" t="n"/>
-      <c r="AA19" s="10" t="n"/>
-      <c r="AB19" s="10" t="n"/>
+      <c r="Y19" s="10" t="n"/>
+      <c r="Z19" s="10" t="n"/>
+      <c r="AA19" s="9" t="n"/>
+      <c r="AB19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>WP4-1</t>
+          <t>WP4-4</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├ W21 — 보완 개발</t>
+          <t xml:space="preserve">  ├ W24 — 프로덕션 배포 + 최종 QA + 프로젝트 종료</t>
         </is>
       </c>
       <c r="C20" s="9" t="n"/>
@@ -3495,11 +3495,11 @@
       <c r="U20" s="9" t="n"/>
       <c r="V20" s="9" t="n"/>
       <c r="W20" s="9" t="n"/>
-      <c r="X20" s="10" t="n"/>
-      <c r="Y20" s="10" t="n"/>
+      <c r="X20" s="9" t="n"/>
+      <c r="Y20" s="9" t="n"/>
       <c r="Z20" s="9" t="n"/>
-      <c r="AA20" s="9" t="n"/>
-      <c r="AB20" s="9" t="n"/>
+      <c r="AA20" s="10" t="n"/>
+      <c r="AB20" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>